<commit_message>
Corrige la ligne d'exemple de pause dans le plan de travail
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sq9w9rcxFpnjt7AwPQjWYF
</commit_message>
<xml_diff>
--- a/production-tournage.xlsx
+++ b/production-tournage.xlsx
@@ -5374,7 +5374,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Feuille de route d'une journée de tournage (8h–20h). Renseigne le n° de séquence pour récupérer décor, personnages et matériel. Horaires modifiables. Une ligne sans séquence sert aux pauses, trajets, installations. Lignes 9-11 et 14 = exemples.</t>
+          <t>Feuille de route d'une journée de tournage (8h–20h). Renseigne le n° de séquence pour récupérer décor, personnages et matériel. Horaires modifiables. Une ligne sans séquence sert aux pauses, trajets, installations. Lignes 9-11 et 17 = exemples.</t>
         </is>
       </c>
     </row>
@@ -5652,11 +5652,7 @@
         <f>IF($C14="","",IFERROR(INDEX('Dépouillement'!$B$6:$B$65,MATCH($C14,'Dépouillement'!$A$6:$A$65,0)),"Séq. introuvable"))</f>
         <v/>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>Pause déjeuner</t>
-        </is>
-      </c>
+      <c r="E14" s="9" t="n"/>
       <c r="F14" s="13">
         <f>IF($C14="","",IFERROR(INDEX('Dépouillement'!$F$6:$F$65,MATCH($C14,'Dépouillement'!$A$6:$A$65,0)),"Séq. introuvable"))</f>
         <v/>
@@ -5665,11 +5661,7 @@
         <f>IF($C14="","",IFERROR(INDEX('Dépouillement'!$J$6:$J$65,MATCH($C14,'Dépouillement'!$A$6:$A$65,0)),"Séq. introuvable"))</f>
         <v/>
       </c>
-      <c r="H14" s="9" t="inlineStr">
-        <is>
-          <t>Exemple – à remplacer</t>
-        </is>
-      </c>
+      <c r="H14" s="9" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="29" t="n">
@@ -5729,7 +5721,11 @@
         <f>IF($C17="","",IFERROR(INDEX('Dépouillement'!$B$6:$B$65,MATCH($C17,'Dépouillement'!$A$6:$A$65,0)),"Séq. introuvable"))</f>
         <v/>
       </c>
-      <c r="E17" s="9" t="n"/>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Pause déjeuner</t>
+        </is>
+      </c>
       <c r="F17" s="13">
         <f>IF($C17="","",IFERROR(INDEX('Dépouillement'!$F$6:$F$65,MATCH($C17,'Dépouillement'!$A$6:$A$65,0)),"Séq. introuvable"))</f>
         <v/>
@@ -5738,7 +5734,11 @@
         <f>IF($C17="","",IFERROR(INDEX('Dépouillement'!$J$6:$J$65,MATCH($C17,'Dépouillement'!$A$6:$A$65,0)),"Séq. introuvable"))</f>
         <v/>
       </c>
-      <c r="H17" s="9" t="n"/>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Exemple – à remplacer</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="29" t="n">

</xml_diff>